<commit_message>
Fix fake merged-word illusion in the 20 new crossword puzzles
Each new puzzle's second across word (e.g. TWO in Emotions) was only
3 letters, placed flush against the tail letters of two unrelated
down words with no blocked cell between them - so row 2 rendered as
one continuous 5-letter run (e.g. "TWONM") even though the game only
treats the first 3 cells as an actual word. Extend the first down
word from 3 to 4 letters and move the second across word to row 3,
so it's followed by genuine blocked cells instead. Verified via a
row-scan check (no across word may touch a filled run without
spanning it exactly) across all 25 puzzles - 0 conflicts, 0
ambiguous runs now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HWaFiXNtTk4AHtDGhZUhLm
</commit_message>
<xml_diff>
--- a/games/cross-word/cw.xlsx
+++ b/games/cross-word/cw.xlsx
@@ -1783,7 +1783,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>COAT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Common house pet that meows</t>
+          <t>Warm outer garment</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SUN</t>
+          <t>SPIN</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Star at the center of our solar system</t>
+          <t>To turn around quickly</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Vehicle with four wheels</t>
+          <t>To burn until black</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>COW</t>
+          <t>CLAW</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Farm animal that gives milk</t>
+          <t>Sharp nail on an animal's paw</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>HAT</t>
+          <t>HEAT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Worn on the head</t>
+          <t>Warmth; high temperature</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>GLUM</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Place to exercise</t>
+          <t>Feeling gloomy or sad</t>
         </is>
       </c>
     </row>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>HEN</t>
+          <t>HORN</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Female chicken</t>
+          <t>Hard growth on an animal's head</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>OWL</t>
+          <t>OVAL</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Nocturnal bird known for hooting</t>
+          <t>Egg-shaped; elliptical</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TOY</t>
+          <t>TIDY</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Plaything for children</t>
+          <t>Neat and organized</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>HOT</t>
+          <t>HUNT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Very warm temperature</t>
+          <t>To search for something</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>USE</t>
+          <t>URGE</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>To make use of something</t>
+          <t>A strong desire to do something</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SAD</t>
+          <t>SEED</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Feeling unhappy</t>
+          <t>What you plant to grow a flower</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D95" t="n">
         <v>0</v>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>CUP</t>
+          <t>CHOP</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Used for drinking</t>
+          <t>To cut into pieces</t>
         </is>
       </c>
     </row>
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D100" t="n">
         <v>0</v>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>CAMP</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Worn on the head, often with a brim</t>
+          <t>Outdoor stay in tents</t>
         </is>
       </c>
     </row>
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ATOM</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Body part with a hand at the end</t>
+          <t>Smallest unit of matter</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>OAR</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Used to row a boat</t>
+          <t>Above; finished</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>NEXT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Mesh used to catch fish</t>
+          <t>Coming right after</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D120" t="n">
         <v>0</v>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>HAM</t>
+          <t>HELM</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Type of cured pork</t>
+          <t>Ship's steering wheel</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>PLAN</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Used for cooking</t>
+          <t>A scheme or intention</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D130" t="n">
         <v>0</v>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NAVY</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>The present moment</t>
+          <t>Sea-based branch of the armed forces</t>
         </is>
       </c>
     </row>
@@ -4331,11 +4331,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>YET</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>To succeed in a game or contest</t>
+          <t>Not now, but eventually</t>
         </is>
       </c>
     </row>

</xml_diff>